<commit_message>
Regenerate database to include missing common subwords (e.g., shill, ills for hills, mast, mats) via a curated whitelist and bump cache version to v42
</commit_message>
<xml_diff>
--- a/seven_letter_words.xlsx
+++ b/seven_letter_words.xlsx
@@ -7754,14 +7754,14 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>ill, bill, sill</t>
+          <t>ill, bill, ills, sill</t>
         </is>
       </c>
       <c r="C408" t="n">
         <v>5</v>
       </c>
       <c r="D408" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="409">
@@ -13226,14 +13226,14 @@
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>his, ill, hill, sill</t>
+          <t>his, ill, hill, ills, sill, shill</t>
         </is>
       </c>
       <c r="C712" t="n">
         <v>5</v>
       </c>
       <c r="D712" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="713">
@@ -13802,14 +13802,14 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>ilk, ill, ski, kill, silk, sill, skill</t>
+          <t>ilk, ill, ski, ills, kill, silk, sill, skill</t>
         </is>
       </c>
       <c r="C744" t="n">
         <v>5</v>
       </c>
       <c r="D744" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="745">
@@ -15170,14 +15170,14 @@
       </c>
       <c r="B820" t="inlineStr">
         <is>
-          <t>ill, mill, sill, slim</t>
+          <t>ill, ills, mill, sill, slim</t>
         </is>
       </c>
       <c r="C820" t="n">
         <v>5</v>
       </c>
       <c r="D820" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="821">
@@ -16646,14 +16646,14 @@
       </c>
       <c r="B902" t="inlineStr">
         <is>
-          <t>ill, lip, sip, lips, lisp, pill, sill, slip, spill</t>
+          <t>ill, lip, sip, ills, lips, lisp, pill, sill, slip, spill</t>
         </is>
       </c>
       <c r="C902" t="n">
         <v>5</v>
       </c>
       <c r="D902" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="903">
@@ -19400,14 +19400,14 @@
       </c>
       <c r="B1055" t="inlineStr">
         <is>
-          <t>ilk, ill, ski, kill, silk, sill, kills</t>
+          <t>ilk, ill, ski, ills, kill, silk, sill, kills</t>
         </is>
       </c>
       <c r="C1055" t="n">
         <v>5</v>
       </c>
       <c r="D1055" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="1056">
@@ -20336,14 +20336,14 @@
       </c>
       <c r="B1107" t="inlineStr">
         <is>
-          <t>ill, its, lit, sit, til, tis, lilt, list, sill, silt, slit, till</t>
+          <t>ill, its, lit, sit, til, tis, ills, lilt, list, sill, silt, slit, till</t>
         </is>
       </c>
       <c r="C1107" t="n">
         <v>5</v>
       </c>
       <c r="D1107" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="1108">
@@ -24044,14 +24044,14 @@
       </c>
       <c r="B1313" t="inlineStr">
         <is>
-          <t>ail, ale, all, ill, lei, lie, sea, ails, isle, leis, lies, sail, sale, seal, sell, sill, aisle</t>
+          <t>ail, ale, all, ill, lei, lie, sea, ails, ills, isle, leis, lies, sail, sale, seal, sell, sill, aisle</t>
         </is>
       </c>
       <c r="C1313" t="n">
         <v>6</v>
       </c>
       <c r="D1313" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="1314">
@@ -29552,14 +29552,14 @@
       </c>
       <c r="B1619" t="inlineStr">
         <is>
-          <t>opt, ore, per, pet, pot, pox, pro, rep, roe, rot, toe, top, poet, pore, port, rope, rote, tore, trope</t>
+          <t>opt, ore, per, pet, pot, pox, pro, rep, roe, rot, toe, top, expo, poet, pore, port, rope, rote, tore, trope</t>
         </is>
       </c>
       <c r="C1619" t="n">
         <v>6</v>
       </c>
       <c r="D1619" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="1620">
@@ -29570,14 +29570,14 @@
       </c>
       <c r="B1620" t="inlineStr">
         <is>
-          <t>pee, pox, see, sex, exes, pees, pose, seep</t>
+          <t>pee, pox, see, sex, exes, expo, pees, pose, seep, expos</t>
         </is>
       </c>
       <c r="C1620" t="n">
         <v>6</v>
       </c>
       <c r="D1620" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1621">
@@ -30740,14 +30740,14 @@
       </c>
       <c r="B1685" t="inlineStr">
         <is>
-          <t>fin, fun, ifs, ins, ion, sin, son, sun, fins, info, ions, onus</t>
+          <t>fin, fun, ifs, ins, ion, sin, son, sun, fins, info, ions, onus, infos</t>
         </is>
       </c>
       <c r="C1685" t="n">
         <v>6</v>
       </c>
       <c r="D1685" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="1686">
@@ -39686,14 +39686,14 @@
       </c>
       <c r="B2182" t="inlineStr">
         <is>
-          <t>ilk, ill, sis, ski, kill, kiss, silk, sill, skis, kills, silks, sills, skill</t>
+          <t>ilk, ill, sis, ski, ills, kill, kiss, silk, sill, skis, kills, silks, sills, skill</t>
         </is>
       </c>
       <c r="C2182" t="n">
         <v>6</v>
       </c>
       <c r="D2182" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2183">
@@ -39848,14 +39848,14 @@
       </c>
       <c r="B2191" t="inlineStr">
         <is>
-          <t>orc, ore, rec, roe, core, orcs, rose, sore, score</t>
+          <t>orc, ore, rec, roe, core, croc, orcs, rose, sore, crocs, score</t>
         </is>
       </c>
       <c r="C2191" t="n">
         <v>6</v>
       </c>
       <c r="D2191" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2192">
@@ -46868,14 +46868,14 @@
       </c>
       <c r="B2581" t="inlineStr">
         <is>
-          <t>con, ion, nor, orc, chic, chin, coin, corn, horn, icon, inch, iron, rich, choir, conch, conic, rhino</t>
+          <t>con, ion, nor, orc, chic, chin, coin, corn, croc, horn, icon, inch, iron, rich, choir, conch, conic, rhino</t>
         </is>
       </c>
       <c r="C2581" t="n">
         <v>7</v>
       </c>
       <c r="D2581" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2582">
@@ -47516,14 +47516,14 @@
       </c>
       <c r="B2617" t="inlineStr">
         <is>
-          <t>cop, elm, mop, pox, come, cope, lope, mole, poem, pole, compel</t>
+          <t>cop, elm, mop, pox, come, cope, expo, lope, mole, poem, pole, compel</t>
         </is>
       </c>
       <c r="C2617" t="n">
         <v>7</v>
       </c>
       <c r="D2617" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2618">
@@ -47570,14 +47570,14 @@
       </c>
       <c r="B2620" t="inlineStr">
         <is>
-          <t>con, eon, nor, one, orc, ore, rec, roe, cone, core, corn, neon, none, once</t>
+          <t>con, eon, nor, one, orc, ore, rec, roe, cone, core, corn, croc, neon, none, once</t>
         </is>
       </c>
       <c r="C2620" t="n">
         <v>7</v>
       </c>
       <c r="D2620" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2621">
@@ -47588,14 +47588,14 @@
       </c>
       <c r="B2621" t="inlineStr">
         <is>
-          <t>con, cot, eon, net, nor, not, one, orc, ore, rec, roe, rot, ten, toe, ton, cent, cone, core, corn, note, once, rent, rote, tern, tone, tore, torn, tenor, toner</t>
+          <t>con, cot, eon, net, nor, not, one, orc, ore, rec, roe, rot, ten, toe, ton, cent, cone, core, corn, croc, note, once, rent, rote, tern, tone, tore, torn, tenor, toner</t>
         </is>
       </c>
       <c r="C2621" t="n">
         <v>7</v>
       </c>
       <c r="D2621" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2622">
@@ -47606,14 +47606,14 @@
       </c>
       <c r="B2622" t="inlineStr">
         <is>
-          <t>cod, con, coo, doc, don, nod, nor, orc, rod, coco, cord, corn, door, odor, condo, donor, condor, cordon</t>
+          <t>cod, con, coo, doc, don, nod, nor, orc, rod, coco, cord, corn, croc, door, odor, condo, donor, condor, cordon</t>
         </is>
       </c>
       <c r="C2622" t="n">
         <v>7</v>
       </c>
       <c r="D2622" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2623">
@@ -50540,14 +50540,14 @@
       </c>
       <c r="B2785" t="inlineStr">
         <is>
-          <t>eel, ere, ore, pee, per, pox, pro, rep, roe, leer, lope, lore, peel, peer, pole, pore, reel, role, rope, elope, expel, repel</t>
+          <t>eel, ere, ore, pee, per, pox, pro, rep, roe, expo, leer, lope, lore, peel, peer, pole, pore, reel, role, rope, elope, expel, repel</t>
         </is>
       </c>
       <c r="C2785" t="n">
         <v>7</v>
       </c>
       <c r="D2785" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2786">
@@ -50558,14 +50558,14 @@
       </c>
       <c r="B2786" t="inlineStr">
         <is>
-          <t>opt, ore, per, pet, pot, pox, pro, rep, roe, rot, set, sex, toe, top, opts, pest, pets, poet, pore, port, pose, post, pots, pros, reps, rest, rope, rose, rote, rots, sore, sort, spot, step, stop, toes, tops, tore, poets, pores, ports, poser, prose, ropes, spore, sport, store, trope, export, poster</t>
+          <t>opt, ore, per, pet, pot, pox, pro, rep, roe, rot, set, sex, toe, top, expo, opts, pest, pets, poet, pore, port, pose, post, pots, pros, reps, rest, rope, rose, rote, rots, sore, sort, spot, step, stop, toes, tops, tore, expos, poets, pores, ports, poser, prose, ropes, spore, sport, store, trope, export, poster</t>
         </is>
       </c>
       <c r="C2786" t="n">
         <v>7</v>
       </c>
       <c r="D2786" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2787">
@@ -50576,14 +50576,14 @@
       </c>
       <c r="B2787" t="inlineStr">
         <is>
-          <t>doe, ode, pee, pod, pox, see, sex, sod, deep, does, dope, dose, exes, odes, peed, pees, pods, pose, seed, seep, dopes, posed, speed, depose, expose</t>
+          <t>doe, ode, pee, pod, pox, see, sex, sod, deep, does, dope, dose, exes, expo, odes, peed, pees, pods, pose, seed, seep, dopes, expos, posed, speed, depose, expose</t>
         </is>
       </c>
       <c r="C2787" t="n">
         <v>7</v>
       </c>
       <c r="D2787" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2788">
@@ -50846,14 +50846,14 @@
       </c>
       <c r="B2802" t="inlineStr">
         <is>
-          <t>ash, fan, fin, has, his, ifs, ins, ion, oaf, sin, son, fans, fins, fish, info, ions, oafs, shin, sofa</t>
+          <t>ash, fan, fin, has, his, ifs, ins, ion, oaf, sin, son, fans, fins, fish, info, ions, oafs, shin, sofa, infos</t>
         </is>
       </c>
       <c r="C2802" t="n">
         <v>7</v>
       </c>
       <c r="D2802" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2803">
@@ -52952,14 +52952,14 @@
       </c>
       <c r="B2919" t="inlineStr">
         <is>
-          <t>ill, ins, lei, lie, nil, sin, sis, isle, leis, lens, less, lies, line, sell, sill, sine, sins, isles, lines, sells, sills</t>
+          <t>ill, ins, lei, lie, nil, sin, sis, ills, isle, leis, lens, less, lies, line, sell, sill, sine, sins, isles, lines, sells, sills</t>
         </is>
       </c>
       <c r="C2919" t="n">
         <v>7</v>
       </c>
       <c r="D2919" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2920">
@@ -53294,14 +53294,14 @@
       </c>
       <c r="B2938" t="inlineStr">
         <is>
-          <t>ail, all, ant, ill, ins, its, lit, nil, nit, sat, sin, sit, tan, til, tin, tis, ails, ants, lain, last, lilt, lint, list, nail, sail, salt, sill, silt, slit, tail, tall, tans, till, tins, nails, saint, satin, slain, slant, snail, stain, stall, still, tails</t>
+          <t>ail, all, ant, ill, ins, its, lit, nil, nit, sat, sin, sit, tan, til, tin, tis, ails, ants, ills, lain, last, lilt, lint, list, nail, sail, salt, sill, silt, slit, tail, tall, tans, till, tins, nails, saint, satin, slain, slant, snail, stain, stall, still, tails</t>
         </is>
       </c>
       <c r="C2938" t="n">
         <v>7</v>
       </c>
       <c r="D2938" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2939">
@@ -56660,14 +56660,14 @@
       </c>
       <c r="B3125" t="inlineStr">
         <is>
-          <t>eon, hen, hex, hip, hoe, hop, ion, nip, one, pen, pie, pin, pox, hone, hope, nope, open, oxen, pine, phone</t>
+          <t>eon, hen, hex, hip, hoe, hop, ion, nip, one, pen, pie, pin, pox, expo, hone, hope, nope, open, oxen, pine, phone</t>
         </is>
       </c>
       <c r="C3125" t="n">
         <v>7</v>
       </c>
       <c r="D3125" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3126">
@@ -59720,14 +59720,14 @@
       </c>
       <c r="B3295" t="inlineStr">
         <is>
-          <t>gel, gin, ill, ins, leg, lei, lie, nil, sin, gels, gill, gins, glen, isle, legs, leis, lens, lies, line, sell, sign, sill, sine, sing, gills, glens, lines, sling, single</t>
+          <t>gel, gin, ill, ins, leg, lei, lie, nil, sin, gels, gill, gins, glen, ills, isle, legs, leis, lens, lies, line, sell, sign, sill, sine, sing, gills, glens, lines, sling, single</t>
         </is>
       </c>
       <c r="C3295" t="n">
         <v>7</v>
       </c>
       <c r="D3295" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3296">
@@ -60422,14 +60422,14 @@
       </c>
       <c r="B3334" t="inlineStr">
         <is>
-          <t>die, elk, ilk, ill, kid, led, lei, lid, lie, ski, deli, dell, desk, dies, dike, dill, disk, elks, idle, isle, kids, kill, leis, lids, lied, lies, like, sell, side, silk, sill, skid, sled, slid, delis, dikes, dills, idles, kills, liked, likes, skill, slide, killed</t>
+          <t>die, elk, ilk, ill, kid, led, lei, lid, lie, ski, deli, dell, desk, dies, dike, dill, disk, elks, idle, ills, isle, kids, kill, leis, lids, lied, lies, like, sell, side, silk, sill, skid, sled, slid, delis, dikes, dills, idles, kills, liked, likes, skill, slide, killed</t>
         </is>
       </c>
       <c r="C3334" t="n">
         <v>7</v>
       </c>
       <c r="D3334" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3335">

</xml_diff>